<commit_message>
turned screener into a function and started trying to solve auto auth issue
</commit_message>
<xml_diff>
--- a/screener/daily_screener_signals/2024-11-05.xlsx
+++ b/screener/daily_screener_signals/2024-11-05.xlsx
@@ -16,7 +16,10 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="2">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+    <numFmt numFmtId="165" formatCode="YYYY-MM-DD"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -55,11 +58,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -425,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:R1"/>
+  <dimension ref="A1:T19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -491,27 +495,1369 @@
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
+          <t>Time Threshold</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Sell_Time</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
           <t>Market Cap</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Sector</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Float</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Market Capitalization</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Shares Float</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ATUS</t>
+        </is>
+      </c>
+      <c r="E2" t="n">
+        <v>2.671122101218081</v>
+      </c>
+      <c r="F2" t="n">
+        <v>10.34108939682302</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0.0538223938223939</v>
+      </c>
+      <c r="H2" t="n">
+        <v>2.34</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="J2" t="n">
+        <v>0.03743744995947515</v>
+      </c>
+      <c r="K2" t="n">
+        <v>2.938234311339889</v>
+      </c>
+      <c r="L2" t="n">
+        <v>2.537565996157177</v>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P2" t="n">
+        <v>1050120000</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Communication Services</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>204860000</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>1050.12M</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>204.86M</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>TIGR</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>6.692448416116755</v>
+      </c>
+      <c r="F3" t="n">
+        <v>13.45755850255508</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.08874801901743273</v>
+      </c>
+      <c r="H3" t="n">
+        <v>6.38</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0.01494221453529324</v>
+      </c>
+      <c r="K3" t="n">
+        <v>7.36169325772843</v>
+      </c>
+      <c r="L3" t="n">
+        <v>6.357825995310917</v>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>1127160000</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="R3" t="n">
+        <v>150250000</v>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>1127.16M</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>150.25M</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>13</v>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>YUMC</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>49.13155673217616</v>
+      </c>
+      <c r="F4" t="n">
+        <v>6.282113389224454</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.1254633269684376</v>
+      </c>
+      <c r="H4" t="n">
+        <v>48.3</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0.002035351750507637</v>
+      </c>
+      <c r="K4" t="n">
+        <v>54.04471240539377</v>
+      </c>
+      <c r="L4" t="n">
+        <v>46.67497889556735</v>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P4" t="n">
+        <v>16682700000</v>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="R4" t="n">
+        <v>368470000</v>
+      </c>
+      <c r="S4" t="inlineStr">
+        <is>
+          <t>16682.7M</t>
+        </is>
+      </c>
+      <c r="T4" t="inlineStr">
+        <is>
+          <t>368.47M</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>15</v>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>FCEL</t>
+        </is>
+      </c>
+      <c r="E5" t="n">
+        <v>0.3953867336066365</v>
+      </c>
+      <c r="F5" t="n">
+        <v>21.38241013634435</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0.2144927536231885</v>
+      </c>
+      <c r="H5" t="n">
+        <v>0.3801</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>10:00:00</t>
+        </is>
+      </c>
+      <c r="J5" t="n">
+        <v>0.2529169329679339</v>
+      </c>
+      <c r="K5" t="n">
+        <v>0.4349254069673001</v>
+      </c>
+      <c r="L5" t="n">
+        <v>0.3756173969263046</v>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P5" t="n">
+        <v>180260000</v>
+      </c>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="R5" t="n">
+        <v>554410000</v>
+      </c>
+      <c r="S5" t="inlineStr">
+        <is>
+          <t>180.26M</t>
+        </is>
+      </c>
+      <c r="T5" t="inlineStr">
+        <is>
+          <t>554.41M</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>FSLR</t>
+        </is>
+      </c>
+      <c r="E6" t="n">
+        <v>214.2514265827297</v>
+      </c>
+      <c r="F6" t="n">
+        <v>10.4930166111947</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0.12486904974832</v>
+      </c>
+      <c r="H6" t="n">
+        <v>211.62</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J6" t="n">
+        <v>0.0004667413496142422</v>
+      </c>
+      <c r="K6" t="n">
+        <v>235.6765692410027</v>
+      </c>
+      <c r="L6" t="n">
+        <v>203.5388552535933</v>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>21008560000</v>
+      </c>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="R6" t="n">
+        <v>101330000</v>
+      </c>
+      <c r="S6" t="inlineStr">
+        <is>
+          <t>21008.56M</t>
+        </is>
+      </c>
+      <c r="T6" t="inlineStr">
+        <is>
+          <t>101.33M</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>14</v>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>NTR</t>
+        </is>
+      </c>
+      <c r="E7" t="n">
+        <v>50.85398113186056</v>
+      </c>
+      <c r="F7" t="n">
+        <v>7.870470245047154</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0.08205987021142964</v>
+      </c>
+      <c r="H7" t="n">
+        <v>50.753462</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>0.001966414384366634</v>
+      </c>
+      <c r="K7" t="n">
+        <v>55.93937924504661</v>
+      </c>
+      <c r="L7" t="n">
+        <v>48.31128207526753</v>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P7" t="n">
+        <v>23407100000</v>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>Basic Materials</t>
+        </is>
+      </c>
+      <c r="R7" t="n">
+        <v>494560000</v>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>23407.1M</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>494.56M</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>8</v>
+      </c>
+      <c r="B8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>NKTR</t>
+        </is>
+      </c>
+      <c r="E8" t="n">
+        <v>1.383960252122809</v>
+      </c>
+      <c r="F8" t="n">
+        <v>13.41802189938773</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0.2003311258278146</v>
+      </c>
+      <c r="H8" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>0.07225641043275154</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.52235627733509</v>
+      </c>
+      <c r="L8" t="n">
+        <v>1.314762239516669</v>
+      </c>
+      <c r="M8" t="inlineStr"/>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>255870000</v>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>Healthcare</t>
+        </is>
+      </c>
+      <c r="R8" t="n">
+        <v>177810000</v>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>255.87M</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>177.81M</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>SLQT</t>
+        </is>
+      </c>
+      <c r="E9" t="n">
+        <v>2.067567482356662</v>
+      </c>
+      <c r="F9" t="n">
+        <v>10.66220692404306</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0.1381909547738694</v>
+      </c>
+      <c r="H9" t="n">
+        <v>2.04</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>0.0483660150652097</v>
+      </c>
+      <c r="K9" t="n">
+        <v>2.274324230592328</v>
+      </c>
+      <c r="L9" t="n">
+        <v>1.964189108238829</v>
+      </c>
+      <c r="M9" t="inlineStr"/>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P9" t="n">
+        <v>336080000</v>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="R9" t="n">
+        <v>135870000</v>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>336.08M</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>135.87M</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ZCAR</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>4.581365065407217</v>
+      </c>
+      <c r="F10" t="n">
+        <v>12.9680708702109</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0.2874396135265702</v>
+      </c>
+      <c r="H10" t="n">
+        <v>4.2651</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>11:00:00</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>0.02182755544959206</v>
+      </c>
+      <c r="K10" t="n">
+        <v>5.039501571947939</v>
+      </c>
+      <c r="L10" t="n">
+        <v>4.352296812136856</v>
+      </c>
+      <c r="M10" t="inlineStr"/>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P10" t="n">
+        <v>5980000</v>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>Industrials</t>
+        </is>
+      </c>
+      <c r="R10" t="n">
+        <v>66550000</v>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>5.98M</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>66.55M</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B11" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>RXT</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>2.515209939133489</v>
+      </c>
+      <c r="F11" t="n">
+        <v>17.29601051367429</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0.06804123711340208</v>
+      </c>
+      <c r="H11" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>11:00:00</t>
+        </is>
+      </c>
+      <c r="J11" t="n">
+        <v>0.03975811261085063</v>
+      </c>
+      <c r="K11" t="n">
+        <v>2.766730933046837</v>
+      </c>
+      <c r="L11" t="n">
+        <v>2.389449442176814</v>
+      </c>
+      <c r="M11" t="inlineStr"/>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P11" t="n">
+        <v>574120000</v>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="R11" t="n">
+        <v>59230000</v>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>574.12M</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>59.23M</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="n">
+        <v>12</v>
+      </c>
+      <c r="B12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>MOS</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>28.6921032519148</v>
+      </c>
+      <c r="F12" t="n">
+        <v>7.206710245838492</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0.08227611940298502</v>
+      </c>
+      <c r="H12" t="n">
+        <v>28.3</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J12" t="n">
+        <v>0.003485279525241022</v>
+      </c>
+      <c r="K12" t="n">
+        <v>31.56131357710628</v>
+      </c>
+      <c r="L12" t="n">
+        <v>27.25749808931906</v>
+      </c>
+      <c r="M12" t="inlineStr"/>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P12" t="n">
+        <v>8291010000</v>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>Basic Materials</t>
+        </is>
+      </c>
+      <c r="R12" t="n">
+        <v>316440000</v>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>8291.01M</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>316.44M</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="n">
+        <v>16</v>
+      </c>
+      <c r="B13" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>XPEV</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>12.30195696665937</v>
+      </c>
+      <c r="F13" t="n">
+        <v>10.94362704044314</v>
+      </c>
+      <c r="G13" t="n">
+        <v>0.1242180518319929</v>
+      </c>
+      <c r="H13" t="n">
+        <v>12.0501</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>0.00812878798641703</v>
+      </c>
+      <c r="K13" t="n">
+        <v>13.53215266332531</v>
+      </c>
+      <c r="L13" t="n">
+        <v>11.6868591183264</v>
+      </c>
+      <c r="M13" t="inlineStr"/>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P13" t="n">
+        <v>8365370000.000001</v>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="R13" t="n">
+        <v>765160000</v>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>8365.37M</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>765.16M</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B14" t="n">
+        <v>0</v>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>FTCI</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>0.6013632334314455</v>
+      </c>
+      <c r="F14" t="n">
+        <v>10.87008835752085</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0.210287443267776</v>
+      </c>
+      <c r="H14" t="n">
+        <v>0.552</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J14" t="n">
+        <v>0.1662888491359688</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0.66149955677459</v>
+      </c>
+      <c r="L14" t="n">
+        <v>0.5712950717598733</v>
+      </c>
+      <c r="M14" t="inlineStr"/>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P14" t="n">
+        <v>84300000</v>
+      </c>
+      <c r="Q14" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="R14" t="n">
+        <v>65060000</v>
+      </c>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>84.3M</t>
+        </is>
+      </c>
+      <c r="T14" t="inlineStr">
+        <is>
+          <t>65.06M</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B15" t="n">
+        <v>0</v>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>FUTU</t>
+        </is>
+      </c>
+      <c r="E15" t="n">
+        <v>99.57189757847354</v>
+      </c>
+      <c r="F15" t="n">
+        <v>13.98681304646174</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0.06430062630480164</v>
+      </c>
+      <c r="H15" t="n">
+        <v>97.20999999999999</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J15" t="n">
+        <v>0.001004299430179977</v>
+      </c>
+      <c r="K15" t="n">
+        <v>109.5290873363209</v>
+      </c>
+      <c r="L15" t="n">
+        <v>94.59330269954987</v>
+      </c>
+      <c r="M15" t="inlineStr"/>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P15" t="n">
+        <v>8631010000</v>
+      </c>
+      <c r="Q15" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
+      <c r="R15" t="n">
+        <v>87310000</v>
+      </c>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>8631.01M</t>
+        </is>
+      </c>
+      <c r="T15" t="inlineStr">
+        <is>
+          <t>87.31M</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="n">
+        <v>11</v>
+      </c>
+      <c r="B16" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>DELL</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>134.2080352624965</v>
+      </c>
+      <c r="F16" t="n">
+        <v>8.913273135852814</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0.09179404666130339</v>
+      </c>
+      <c r="H16" t="n">
+        <v>130.14</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J16" t="n">
+        <v>0.0007451118690800497</v>
+      </c>
+      <c r="K16" t="n">
+        <v>147.6288387887462</v>
+      </c>
+      <c r="L16" t="n">
+        <v>127.4976334993717</v>
+      </c>
+      <c r="M16" t="inlineStr"/>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P16" t="n">
+        <v>91543310000</v>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="R16" t="n">
+        <v>308390000</v>
+      </c>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>91543.31M</t>
+        </is>
+      </c>
+      <c r="T16" t="inlineStr">
+        <is>
+          <t>308.39M</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" t="n">
+        <v>0</v>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>SHW</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>376.8005395255976</v>
+      </c>
+      <c r="F17" t="n">
+        <v>20.15279414349347</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0.0643550624133148</v>
+      </c>
+      <c r="H17" t="n">
+        <v>374.25</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J17" t="n">
+        <v>0.0002653924013110565</v>
+      </c>
+      <c r="K17" t="n">
+        <v>414.4805934781573</v>
+      </c>
+      <c r="L17" t="n">
+        <v>357.9605125493177</v>
+      </c>
+      <c r="M17" t="inlineStr"/>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P17" t="n">
+        <v>96300250000</v>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Basic Materials</t>
+        </is>
+      </c>
+      <c r="R17" t="n">
+        <v>231780000</v>
+      </c>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>96300.25M</t>
+        </is>
+      </c>
+      <c r="T17" t="inlineStr">
+        <is>
+          <t>231.78M</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B18" t="n">
+        <v>0</v>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SEDG</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>18.45613106859861</v>
+      </c>
+      <c r="F18" t="n">
+        <v>12.05732448994231</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0.1233842538190365</v>
+      </c>
+      <c r="H18" t="n">
+        <v>18.25</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J18" t="n">
+        <v>0.005418253675611391</v>
+      </c>
+      <c r="K18" t="n">
+        <v>20.30174417545847</v>
+      </c>
+      <c r="L18" t="n">
+        <v>17.53332451516868</v>
+      </c>
+      <c r="M18" t="inlineStr"/>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P18" t="n">
+        <v>974670000</v>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="R18" t="n">
+        <v>56620000</v>
+      </c>
+      <c r="S18" t="inlineStr">
+        <is>
+          <t>974.67M</t>
+        </is>
+      </c>
+      <c r="T18" t="inlineStr">
+        <is>
+          <t>56.62M</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>45600</v>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>NIO</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>5.215035382317161</v>
+      </c>
+      <c r="F19" t="n">
+        <v>6.4952106436749</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0.05999999999999996</v>
+      </c>
+      <c r="H19" t="n">
+        <v>5.15</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>09:30:00</t>
+        </is>
+      </c>
+      <c r="J19" t="n">
+        <v>0.01917532531784428</v>
+      </c>
+      <c r="K19" t="n">
+        <v>5.736538920548877</v>
+      </c>
+      <c r="L19" t="n">
+        <v>4.954283613201303</v>
+      </c>
+      <c r="M19" t="inlineStr"/>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>12:30:00</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>15:30:00</t>
+        </is>
+      </c>
+      <c r="P19" t="n">
+        <v>9888690000</v>
+      </c>
+      <c r="Q19" t="inlineStr">
+        <is>
+          <t>Consumer Cyclical</t>
+        </is>
+      </c>
+      <c r="R19" t="n">
+        <v>1923830000</v>
+      </c>
+      <c r="S19" t="inlineStr">
+        <is>
+          <t>9888.69M</t>
+        </is>
+      </c>
+      <c r="T19" t="inlineStr">
+        <is>
+          <t>1923.83M</t>
         </is>
       </c>
     </row>

</xml_diff>